<commit_message>
fully implemented forcedecks into Model_1
</commit_message>
<xml_diff>
--- a/HRV_and_Readiness3_audit.xlsx
+++ b/HRV_and_Readiness3_audit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a832f6e089c31e67/Desktop/RegAnProject/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="11_284D8FE730BC1B9A58B3BB3526101A939CBF0475" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00EC4760-B217-4080-B537-88A8B8D33B36}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="11_284D8FE730BC1B9A58B3BB3526101A939CBF0475" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1206C1F4-8A74-4D26-B103-E1C97B09232B}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="3860" yWindow="3110" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variable Summary" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="92">
   <si>
     <t>variable</t>
   </si>
@@ -297,12 +297,6 @@
   </si>
   <si>
     <t>HRV and Readiness3 audit covers 16 athletes from 2026-01-23 to 2026-06-15. Mean observations per athlete: 106.31 (range 60–139). Mean gap between observations: 1.28 days (range 1.0–19.0 days).</t>
-  </si>
-  <si>
-    <t>correct</t>
-  </si>
-  <si>
-    <t>y</t>
   </si>
 </sst>
 </file>
@@ -310,7 +304,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -343,7 +337,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -646,13 +640,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N62"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -683,11 +677,8 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="N1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -718,11 +709,8 @@
       <c r="J2" t="s">
         <v>12</v>
       </c>
-      <c r="N2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -753,11 +741,8 @@
       <c r="J3" t="s">
         <v>12</v>
       </c>
-      <c r="N3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -788,11 +773,8 @@
       <c r="J4" t="s">
         <v>16</v>
       </c>
-      <c r="N4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -823,11 +805,8 @@
       <c r="J5" t="s">
         <v>16</v>
       </c>
-      <c r="N5" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -858,11 +837,8 @@
       <c r="J6" t="s">
         <v>20</v>
       </c>
-      <c r="N6" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -893,11 +869,8 @@
       <c r="J7" t="s">
         <v>22</v>
       </c>
-      <c r="N7" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -928,11 +901,8 @@
       <c r="J8" t="s">
         <v>20</v>
       </c>
-      <c r="N8" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -963,11 +933,8 @@
       <c r="J9" t="s">
         <v>16</v>
       </c>
-      <c r="N9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -998,11 +965,8 @@
       <c r="J10" t="s">
         <v>16</v>
       </c>
-      <c r="N10" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -1033,11 +997,8 @@
       <c r="J11" t="s">
         <v>16</v>
       </c>
-      <c r="N11" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -1068,11 +1029,8 @@
       <c r="J12" t="s">
         <v>16</v>
       </c>
-      <c r="N12" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1103,11 +1061,8 @@
       <c r="J13" t="s">
         <v>29</v>
       </c>
-      <c r="N13" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -1138,11 +1093,8 @@
       <c r="J14" t="s">
         <v>22</v>
       </c>
-      <c r="N14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>31</v>
       </c>
@@ -1173,11 +1125,8 @@
       <c r="J15" t="s">
         <v>22</v>
       </c>
-      <c r="N15" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -1208,11 +1157,8 @@
       <c r="J16" t="s">
         <v>22</v>
       </c>
-      <c r="N16" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>33</v>
       </c>
@@ -1243,11 +1189,8 @@
       <c r="J17" t="s">
         <v>22</v>
       </c>
-      <c r="N17" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -1278,11 +1221,8 @@
       <c r="J18" t="s">
         <v>22</v>
       </c>
-      <c r="N18" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -1313,11 +1253,8 @@
       <c r="J19" t="s">
         <v>22</v>
       </c>
-      <c r="N19" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -1348,11 +1285,8 @@
       <c r="J20" t="s">
         <v>16</v>
       </c>
-      <c r="N20" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -1383,11 +1317,8 @@
       <c r="J21" t="s">
         <v>16</v>
       </c>
-      <c r="N21" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>38</v>
       </c>
@@ -1418,11 +1349,8 @@
       <c r="J22" t="s">
         <v>20</v>
       </c>
-      <c r="N22" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>39</v>
       </c>
@@ -1453,11 +1381,8 @@
       <c r="J23" t="s">
         <v>20</v>
       </c>
-      <c r="N23" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>40</v>
       </c>
@@ -1488,11 +1413,8 @@
       <c r="J24" t="s">
         <v>29</v>
       </c>
-      <c r="N24" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>41</v>
       </c>
@@ -1523,11 +1445,8 @@
       <c r="J25" t="s">
         <v>29</v>
       </c>
-      <c r="N25" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>42</v>
       </c>
@@ -1558,11 +1477,8 @@
       <c r="J26" t="s">
         <v>43</v>
       </c>
-      <c r="N26" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>44</v>
       </c>
@@ -1593,11 +1509,8 @@
       <c r="J27" t="s">
         <v>20</v>
       </c>
-      <c r="N27" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>45</v>
       </c>
@@ -1628,11 +1541,8 @@
       <c r="J28" t="s">
         <v>16</v>
       </c>
-      <c r="N28" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>46</v>
       </c>
@@ -1663,11 +1573,8 @@
       <c r="J29" t="s">
         <v>16</v>
       </c>
-      <c r="N29" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>47</v>
       </c>
@@ -1698,11 +1605,8 @@
       <c r="J30" t="s">
         <v>16</v>
       </c>
-      <c r="N30" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>48</v>
       </c>
@@ -1733,11 +1637,8 @@
       <c r="J31" t="s">
         <v>16</v>
       </c>
-      <c r="N31" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>49</v>
       </c>
@@ -1768,11 +1669,8 @@
       <c r="J32" t="s">
         <v>16</v>
       </c>
-      <c r="N32" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>50</v>
       </c>
@@ -1803,11 +1701,8 @@
       <c r="J33" t="s">
         <v>16</v>
       </c>
-      <c r="N33" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>51</v>
       </c>
@@ -1838,11 +1733,8 @@
       <c r="J34" t="s">
         <v>16</v>
       </c>
-      <c r="N34" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>52</v>
       </c>
@@ -1873,11 +1765,8 @@
       <c r="J35" t="s">
         <v>16</v>
       </c>
-      <c r="N35" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>53</v>
       </c>
@@ -1908,11 +1797,8 @@
       <c r="J36" t="s">
         <v>20</v>
       </c>
-      <c r="N36" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>54</v>
       </c>
@@ -1943,11 +1829,8 @@
       <c r="J37" t="s">
         <v>20</v>
       </c>
-      <c r="N37" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>55</v>
       </c>
@@ -1978,11 +1861,8 @@
       <c r="J38" t="s">
         <v>20</v>
       </c>
-      <c r="N38" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>56</v>
       </c>
@@ -2013,11 +1893,8 @@
       <c r="J39" t="s">
         <v>20</v>
       </c>
-      <c r="N39" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>57</v>
       </c>
@@ -2048,11 +1925,8 @@
       <c r="J40" t="s">
         <v>20</v>
       </c>
-      <c r="N40" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>58</v>
       </c>
@@ -2083,11 +1957,8 @@
       <c r="J41" t="s">
         <v>20</v>
       </c>
-      <c r="N41" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>59</v>
       </c>
@@ -2118,11 +1989,8 @@
       <c r="J42" t="s">
         <v>20</v>
       </c>
-      <c r="N42" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>60</v>
       </c>
@@ -2153,11 +2021,8 @@
       <c r="J43" t="s">
         <v>12</v>
       </c>
-      <c r="N43" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>61</v>
       </c>
@@ -2188,11 +2053,8 @@
       <c r="J44" t="s">
         <v>22</v>
       </c>
-      <c r="N44" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>62</v>
       </c>
@@ -2223,11 +2085,8 @@
       <c r="J45" t="s">
         <v>29</v>
       </c>
-      <c r="N45" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>63</v>
       </c>
@@ -2258,11 +2117,8 @@
       <c r="J46" t="s">
         <v>29</v>
       </c>
-      <c r="N46" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>64</v>
       </c>
@@ -2293,11 +2149,8 @@
       <c r="J47" t="s">
         <v>29</v>
       </c>
-      <c r="N47" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>65</v>
       </c>
@@ -2328,11 +2181,8 @@
       <c r="J48" t="s">
         <v>43</v>
       </c>
-      <c r="N48" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>66</v>
       </c>
@@ -2363,11 +2213,8 @@
       <c r="J49" t="s">
         <v>20</v>
       </c>
-      <c r="N49" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>67</v>
       </c>
@@ -2398,11 +2245,8 @@
       <c r="J50" t="s">
         <v>20</v>
       </c>
-      <c r="N50" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>68</v>
       </c>
@@ -2433,11 +2277,8 @@
       <c r="J51" t="s">
         <v>20</v>
       </c>
-      <c r="N51" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>69</v>
       </c>
@@ -2468,11 +2309,8 @@
       <c r="J52" t="s">
         <v>20</v>
       </c>
-      <c r="N52" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>70</v>
       </c>
@@ -2503,11 +2341,8 @@
       <c r="J53" t="s">
         <v>20</v>
       </c>
-      <c r="N53" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>71</v>
       </c>
@@ -2538,11 +2373,8 @@
       <c r="J54" t="s">
         <v>20</v>
       </c>
-      <c r="N54" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>72</v>
       </c>
@@ -2573,11 +2405,8 @@
       <c r="J55" t="s">
         <v>20</v>
       </c>
-      <c r="N55" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>73</v>
       </c>
@@ -2608,11 +2437,8 @@
       <c r="J56" t="s">
         <v>22</v>
       </c>
-      <c r="N56" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>74</v>
       </c>
@@ -2643,11 +2469,8 @@
       <c r="J57" t="s">
         <v>22</v>
       </c>
-      <c r="N57" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>75</v>
       </c>
@@ -2678,11 +2501,8 @@
       <c r="J58" t="s">
         <v>22</v>
       </c>
-      <c r="N58" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>76</v>
       </c>
@@ -2713,11 +2533,8 @@
       <c r="J59" t="s">
         <v>22</v>
       </c>
-      <c r="N59" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>77</v>
       </c>
@@ -2748,11 +2565,8 @@
       <c r="J60" t="s">
         <v>22</v>
       </c>
-      <c r="N60" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>78</v>
       </c>
@@ -2783,11 +2597,8 @@
       <c r="J61" t="s">
         <v>12</v>
       </c>
-      <c r="N61" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>79</v>
       </c>
@@ -2817,9 +2628,6 @@
       </c>
       <c r="J62" t="s">
         <v>12</v>
-      </c>
-      <c r="N62" t="s">
-        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -2831,6 +2639,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">

</xml_diff>